<commit_message>
Lich tuan xem theo ngay/buoi nhom theo vi tri; giu xe la flag + popup chon nguoi
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DangKyCa-CoSo3.xlsx
+++ b/DangKyCa-CoSo3.xlsx
@@ -559,7 +559,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Định mức mỗi buổi:  Pha chế 2  ·  Phục vụ 2–3  ·  Giữ xe 1</t>
+          <t>Định mức mỗi buổi:  Pha chế 2  ·  Phục vụ 2–3   (người giữ xe do chủ quán chọn trong app)</t>
         </is>
       </c>
     </row>
@@ -1083,175 +1083,175 @@
   </sheetData>
   <conditionalFormatting sqref="C5:C20">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
-      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D20">
     <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="4" dxfId="1">
-      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:E20">
     <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="1">
-      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F20">
     <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="8" dxfId="1">
-      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G20">
     <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="1">
-      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H20">
     <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="12" dxfId="1">
-      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I20">
     <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
-      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="14" dxfId="1">
-      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J20">
     <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
-      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="16" dxfId="1">
-      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K20">
     <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
-      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="18" dxfId="1">
-      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L20">
     <cfRule type="expression" priority="19" dxfId="0" stopIfTrue="1">
-      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="20" dxfId="1">
-      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M5:M20">
     <cfRule type="expression" priority="21" dxfId="0" stopIfTrue="1">
-      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="22" dxfId="1">
-      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:N20">
     <cfRule type="expression" priority="23" dxfId="0" stopIfTrue="1">
-      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="24" dxfId="1">
-      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O20">
     <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
-      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="26" dxfId="1">
-      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P20">
     <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
-      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="28" dxfId="1">
-      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q20">
     <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
-      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="30" dxfId="1">
-      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:R20">
     <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
-      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="32" dxfId="1">
-      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5:S20">
     <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
-      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="34" dxfId="1">
-      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:T20">
     <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
-      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="36" dxfId="1">
-      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U5:U20">
     <cfRule type="expression" priority="37" dxfId="0" stopIfTrue="1">
-      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="38" dxfId="1">
-      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:V20">
     <cfRule type="expression" priority="39" dxfId="0" stopIfTrue="1">
-      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="40" dxfId="1">
-      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W20">
     <cfRule type="expression" priority="41" dxfId="0" stopIfTrue="1">
-      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
     <cfRule type="expression" priority="42" dxfId="1">
-      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,IF($B5="Giữ xe",1,99))))</formula>
+      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="B5:B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Pha chế,Phục vụ,Giữ xe"</formula1>
+      <formula1>"Pha chế,Phục vụ"</formula1>
     </dataValidation>
     <dataValidation sqref="C5:W20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
@@ -1337,10 +1337,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E5" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!C$5:C$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
@@ -1361,10 +1357,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E6" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!D$5:D$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -1385,10 +1377,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E7" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!E$5:E$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1409,10 +1397,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E8" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!F$5:F$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1433,10 +1417,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E9" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!G$5:G$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1457,10 +1437,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E10" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!H$5:H$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1481,10 +1457,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E11" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!I$5:I$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1505,10 +1477,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E12" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!J$5:J$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -1529,10 +1497,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E13" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!K$5:K$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
@@ -1553,10 +1517,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E14" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!L$5:L$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -1577,10 +1537,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E15" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!M$5:M$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -1601,10 +1557,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E16" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!N$5:N$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
@@ -1625,10 +1577,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E17" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!O$5:O$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -1649,10 +1597,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E18" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!P$5:P$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -1673,10 +1617,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E19" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!Q$5:Q$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -1697,10 +1637,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E20" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!R$5:R$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -1721,10 +1657,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E21" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!S$5:S$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -1745,10 +1677,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E22" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!T$5:T$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -1769,10 +1697,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&amp;"/3"</f>
         <v/>
       </c>
-      <c r="E23" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!U$5:U$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -1793,10 +1717,6 @@
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&amp;"/2"</f>
         <v/>
       </c>
-      <c r="E24" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!V$5:V$20,"x")&amp;"/1"</f>
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -1815,10 +1735,6 @@
       </c>
       <c r="D25" s="8">
         <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-      <c r="E25" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!W$5:W$20,"x")&amp;"/1"</f>
         <v/>
       </c>
     </row>
@@ -1833,309 +1749,204 @@
       <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&gt;=3</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5">
+  <conditionalFormatting sqref="C6">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!C$5:C$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D6">
     <cfRule type="expression" priority="4" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7">
     <cfRule type="expression" priority="5" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D7">
     <cfRule type="expression" priority="6" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!D$5:D$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C8">
     <cfRule type="expression" priority="7" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D8">
     <cfRule type="expression" priority="8" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E7">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
     <cfRule type="expression" priority="9" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!E$5:E$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D9">
     <cfRule type="expression" priority="10" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D8">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10">
     <cfRule type="expression" priority="11" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D10">
     <cfRule type="expression" priority="12" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!F$5:F$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C11">
     <cfRule type="expression" priority="13" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D9">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D11">
     <cfRule type="expression" priority="14" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12">
     <cfRule type="expression" priority="15" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!G$5:G$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D12">
     <cfRule type="expression" priority="16" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D10">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C13">
     <cfRule type="expression" priority="17" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E10">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D13">
     <cfRule type="expression" priority="18" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!H$5:H$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C14">
     <cfRule type="expression" priority="19" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D11">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
     <cfRule type="expression" priority="20" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E11">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C15">
     <cfRule type="expression" priority="21" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!I$5:I$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C12">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D15">
     <cfRule type="expression" priority="22" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D12">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C16">
     <cfRule type="expression" priority="23" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E12">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D16">
     <cfRule type="expression" priority="24" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!J$5:J$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C17">
     <cfRule type="expression" priority="25" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D13">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D17">
     <cfRule type="expression" priority="26" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E13">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C18">
     <cfRule type="expression" priority="27" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!K$5:K$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C14">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D18">
     <cfRule type="expression" priority="28" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D14">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C19">
     <cfRule type="expression" priority="29" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E14">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D19">
     <cfRule type="expression" priority="30" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!L$5:L$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C15">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C20">
     <cfRule type="expression" priority="31" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D15">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D20">
     <cfRule type="expression" priority="32" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E15">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C21">
     <cfRule type="expression" priority="33" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!M$5:M$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D21">
     <cfRule type="expression" priority="34" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C22">
     <cfRule type="expression" priority="35" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E16">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D22">
     <cfRule type="expression" priority="36" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!N$5:N$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C23">
     <cfRule type="expression" priority="37" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23">
     <cfRule type="expression" priority="38" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E17">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&gt;=3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C24">
     <cfRule type="expression" priority="39" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!O$5:O$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D24">
     <cfRule type="expression" priority="40" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D18">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C25">
     <cfRule type="expression" priority="41" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E18">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&gt;=2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D25">
     <cfRule type="expression" priority="42" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!P$5:P$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
-    <cfRule type="expression" priority="43" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19">
-    <cfRule type="expression" priority="44" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E19">
-    <cfRule type="expression" priority="45" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!Q$5:Q$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
-    <cfRule type="expression" priority="46" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
-    <cfRule type="expression" priority="47" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E20">
-    <cfRule type="expression" priority="48" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!R$5:R$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
-    <cfRule type="expression" priority="49" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D21">
-    <cfRule type="expression" priority="50" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E21">
-    <cfRule type="expression" priority="51" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!S$5:S$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="expression" priority="52" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22">
-    <cfRule type="expression" priority="53" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E22">
-    <cfRule type="expression" priority="54" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!T$5:T$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
-    <cfRule type="expression" priority="55" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="expression" priority="56" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23">
-    <cfRule type="expression" priority="57" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!U$5:U$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
-    <cfRule type="expression" priority="58" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D24">
-    <cfRule type="expression" priority="59" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E24">
-    <cfRule type="expression" priority="60" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!V$5:V$20,"x")&gt;=1</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
-    <cfRule type="expression" priority="61" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&gt;=2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D25">
-    <cfRule type="expression" priority="62" dxfId="0">
       <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&gt;=3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E25">
-    <cfRule type="expression" priority="63" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Giữ xe",'Đăng ký'!W$5:W$20,"x")&gt;=1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Dang ky buoi ranh + tu xep ca can bang (dam bao ca toi thieu, uu tien nguoi it ca); form doi sang availability
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DangKyCa-CoSo3.xlsx
+++ b/DangKyCa-CoSo3.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Đăng ký" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Còn chỗ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Số bạn rảnh" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -141,14 +141,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F6C6C0"/>
+          <fgColor rgb="00CDE9D5"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00CDE9D5"/>
+          <fgColor rgb="00F6C6C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -545,21 +545,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ĐĂNG KÝ CA LÀM — CƠ SỞ 3</t>
+          <t>ĐĂNG KÝ BUỔI RẢNH — CƠ SỞ 3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Điền chữ  x  vào buổi bạn ĐI LÀM ĐƯỢC. Ai điền trước được ưu tiên. Ô chuyển ĐỎ = buổi đó đã đủ người → hãy chọn buổi/ngày khác. Ô XANH = đã nhận chỗ.</t>
+          <t>Điền chữ  x  vào MỌI buổi bạn ĐI LÀM ĐƯỢC (rảnh). Càng đăng ký nhiều buổi rảnh, càng dễ được xếp đủ ca. App sẽ tự chia cân bằng và ưu tiên người ít ca — không phải ai điền trước.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Định mức mỗi buổi:  Pha chế 2  ·  Phục vụ 2–3   (người giữ xe do chủ quán chọn trong app)</t>
+          <t>Ô XANH = đã đăng ký rảnh.  Người giữ xe do chủ quán chọn trong app.</t>
         </is>
       </c>
     </row>
@@ -1082,171 +1082,108 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5:C20">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>AND(C5="x",COUNTIFS($B$5:$B5,$B5,C$5:C5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>LOWER(C5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D20">
-    <cfRule type="expression" priority="3" dxfId="0" stopIfTrue="1">
-      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>AND(D5="x",COUNTIFS($B$5:$B5,$B5,D$5:D5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>LOWER(D5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:E20">
-    <cfRule type="expression" priority="5" dxfId="0" stopIfTrue="1">
-      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="1">
-      <formula>AND(E5="x",COUNTIFS($B$5:$B5,$B5,E$5:E5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>LOWER(E5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:F20">
-    <cfRule type="expression" priority="7" dxfId="0" stopIfTrue="1">
-      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="8" dxfId="1">
-      <formula>AND(F5="x",COUNTIFS($B$5:$B5,$B5,F$5:F5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="4" dxfId="0">
+      <formula>LOWER(F5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:G20">
-    <cfRule type="expression" priority="9" dxfId="0" stopIfTrue="1">
-      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="10" dxfId="1">
-      <formula>AND(G5="x",COUNTIFS($B$5:$B5,$B5,G$5:G5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="5" dxfId="0">
+      <formula>LOWER(G5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H20">
-    <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12" dxfId="1">
-      <formula>AND(H5="x",COUNTIFS($B$5:$B5,$B5,H$5:H5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="6" dxfId="0">
+      <formula>LOWER(H5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I20">
-    <cfRule type="expression" priority="13" dxfId="0" stopIfTrue="1">
-      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="14" dxfId="1">
-      <formula>AND(I5="x",COUNTIFS($B$5:$B5,$B5,I$5:I5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="7" dxfId="0">
+      <formula>LOWER(I5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J5:J20">
-    <cfRule type="expression" priority="15" dxfId="0" stopIfTrue="1">
-      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="16" dxfId="1">
-      <formula>AND(J5="x",COUNTIFS($B$5:$B5,$B5,J$5:J5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="8" dxfId="0">
+      <formula>LOWER(J5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:K20">
-    <cfRule type="expression" priority="17" dxfId="0" stopIfTrue="1">
-      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="18" dxfId="1">
-      <formula>AND(K5="x",COUNTIFS($B$5:$B5,$B5,K$5:K5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="9" dxfId="0">
+      <formula>LOWER(K5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:L20">
-    <cfRule type="expression" priority="19" dxfId="0" stopIfTrue="1">
-      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="20" dxfId="1">
-      <formula>AND(L5="x",COUNTIFS($B$5:$B5,$B5,L$5:L5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="10" dxfId="0">
+      <formula>LOWER(L5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M5:M20">
-    <cfRule type="expression" priority="21" dxfId="0" stopIfTrue="1">
-      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="22" dxfId="1">
-      <formula>AND(M5="x",COUNTIFS($B$5:$B5,$B5,M$5:M5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="11" dxfId="0">
+      <formula>LOWER(M5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:N20">
-    <cfRule type="expression" priority="23" dxfId="0" stopIfTrue="1">
-      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="24" dxfId="1">
-      <formula>AND(N5="x",COUNTIFS($B$5:$B5,$B5,N$5:N5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="12" dxfId="0">
+      <formula>LOWER(N5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O5:O20">
-    <cfRule type="expression" priority="25" dxfId="0" stopIfTrue="1">
-      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="26" dxfId="1">
-      <formula>AND(O5="x",COUNTIFS($B$5:$B5,$B5,O$5:O5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="13" dxfId="0">
+      <formula>LOWER(O5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:P20">
-    <cfRule type="expression" priority="27" dxfId="0" stopIfTrue="1">
-      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="28" dxfId="1">
-      <formula>AND(P5="x",COUNTIFS($B$5:$B5,$B5,P$5:P5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="14" dxfId="0">
+      <formula>LOWER(P5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q20">
-    <cfRule type="expression" priority="29" dxfId="0" stopIfTrue="1">
-      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30" dxfId="1">
-      <formula>AND(Q5="x",COUNTIFS($B$5:$B5,$B5,Q$5:Q5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="15" dxfId="0">
+      <formula>LOWER(Q5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:R20">
-    <cfRule type="expression" priority="31" dxfId="0" stopIfTrue="1">
-      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="32" dxfId="1">
-      <formula>AND(R5="x",COUNTIFS($B$5:$B5,$B5,R$5:R5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="16" dxfId="0">
+      <formula>LOWER(R5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S5:S20">
-    <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
-      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="34" dxfId="1">
-      <formula>AND(S5="x",COUNTIFS($B$5:$B5,$B5,S$5:S5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="17" dxfId="0">
+      <formula>LOWER(S5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T5:T20">
-    <cfRule type="expression" priority="35" dxfId="0" stopIfTrue="1">
-      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="36" dxfId="1">
-      <formula>AND(T5="x",COUNTIFS($B$5:$B5,$B5,T$5:T5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="18" dxfId="0">
+      <formula>LOWER(T5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U5:U20">
-    <cfRule type="expression" priority="37" dxfId="0" stopIfTrue="1">
-      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="38" dxfId="1">
-      <formula>AND(U5="x",COUNTIFS($B$5:$B5,$B5,U$5:U5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="19" dxfId="0">
+      <formula>LOWER(U5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:V20">
-    <cfRule type="expression" priority="39" dxfId="0" stopIfTrue="1">
-      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="40" dxfId="1">
-      <formula>AND(V5="x",COUNTIFS($B$5:$B5,$B5,V$5:V5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",2,99)))</formula>
+    <cfRule type="expression" priority="20" dxfId="0">
+      <formula>LOWER(V5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W20">
-    <cfRule type="expression" priority="41" dxfId="0" stopIfTrue="1">
-      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&gt;IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="42" dxfId="1">
-      <formula>AND(W5="x",COUNTIFS($B$5:$B5,$B5,W$5:W5,"x")&lt;=IF($B5="Pha chế",2,IF($B5="Phục vụ",3,99)))</formula>
+    <cfRule type="expression" priority="21" dxfId="0">
+      <formula>LOWER(W5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -1267,27 +1204,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>CÒN CHỖ MỖI BUỔI (tự cập nhật)</t>
+          <t>SỐ BẠN RẢNH MỖI BUỔI (tự cập nhật)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Số đang có / định mức. Ô đỏ = đã đủ.</t>
+          <t>Số bạn đăng ký rảnh / định mức cần. Ô ĐỎ = chưa đủ người rảnh → cần thêm bạn đăng ký buổi này.</t>
         </is>
       </c>
     </row>
@@ -1312,11 +1248,6 @@
           <t>Phục vụ</t>
         </is>
       </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Giữ xe</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -1740,213 +1671,213 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C5">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!C$5:C$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!C$5:C$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5">
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6">
-    <cfRule type="expression" priority="3" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6">
-    <cfRule type="expression" priority="4" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7">
-    <cfRule type="expression" priority="5" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="5" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7">
-    <cfRule type="expression" priority="6" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="6" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8">
-    <cfRule type="expression" priority="7" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="7" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D8">
-    <cfRule type="expression" priority="8" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="8" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C9">
-    <cfRule type="expression" priority="9" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="9" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="expression" priority="10" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="10" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10">
-    <cfRule type="expression" priority="11" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="11" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D10">
-    <cfRule type="expression" priority="12" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="12" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" priority="13" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="13" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="expression" priority="14" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="14" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C12">
-    <cfRule type="expression" priority="15" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="15" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12">
-    <cfRule type="expression" priority="16" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="16" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13">
-    <cfRule type="expression" priority="17" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="17" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13">
-    <cfRule type="expression" priority="18" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="18" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14">
-    <cfRule type="expression" priority="19" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="19" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14">
-    <cfRule type="expression" priority="20" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="20" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C15">
-    <cfRule type="expression" priority="21" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="21" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15">
-    <cfRule type="expression" priority="22" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="22" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C16">
-    <cfRule type="expression" priority="23" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="23" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16">
-    <cfRule type="expression" priority="24" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="24" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17">
-    <cfRule type="expression" priority="25" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="25" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17">
-    <cfRule type="expression" priority="26" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="26" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="expression" priority="27" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="27" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="expression" priority="28" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="28" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C19">
-    <cfRule type="expression" priority="29" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="29" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19">
-    <cfRule type="expression" priority="30" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="30" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20">
-    <cfRule type="expression" priority="31" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="31" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D20">
-    <cfRule type="expression" priority="32" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="32" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C21">
-    <cfRule type="expression" priority="33" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="33" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D21">
-    <cfRule type="expression" priority="34" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="34" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C22">
-    <cfRule type="expression" priority="35" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="35" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D22">
-    <cfRule type="expression" priority="36" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="36" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23">
-    <cfRule type="expression" priority="37" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="37" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D23">
-    <cfRule type="expression" priority="38" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="38" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C24">
-    <cfRule type="expression" priority="39" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="39" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D24">
-    <cfRule type="expression" priority="40" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="40" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C25">
-    <cfRule type="expression" priority="41" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&gt;=2</formula>
+    <cfRule type="expression" priority="41" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&lt;2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D25">
-    <cfRule type="expression" priority="42" dxfId="0">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&gt;=3</formula>
+    <cfRule type="expression" priority="42" dxfId="1">
+      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&lt;3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sheet dang ky gon (chi bao ranh/ban, them cot Tong ranh); tranh xep ca toi->sang hom sau
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DangKyCa-CoSo3.xlsx
+++ b/DangKyCa-CoSo3.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Đăng ký" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Số bạn rảnh" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,11 +37,6 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="006B5B4C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
       <color rgb="003A2A1E"/>
     </font>
     <font>
@@ -53,7 +47,11 @@
     <font>
       <b val="1"/>
       <color rgb="009A461C"/>
-      <sz val="14"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009A461C"/>
     </font>
   </fonts>
   <fills count="5">
@@ -70,12 +68,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBF3E6"/>
+        <fgColor rgb="00FBF4E7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3E7D6"/>
+        <fgColor rgb="00F1E4D2"/>
       </patternFill>
     </fill>
   </fills>
@@ -105,18 +103,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,26 +129,18 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00CDE9D5"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F6C6C0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -514,32 +506,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:X22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="8.5" customWidth="1" min="3" max="3"/>
-    <col width="8.5" customWidth="1" min="4" max="4"/>
-    <col width="8.5" customWidth="1" min="5" max="5"/>
-    <col width="8.5" customWidth="1" min="6" max="6"/>
-    <col width="8.5" customWidth="1" min="7" max="7"/>
-    <col width="8.5" customWidth="1" min="8" max="8"/>
-    <col width="8.5" customWidth="1" min="9" max="9"/>
-    <col width="8.5" customWidth="1" min="10" max="10"/>
-    <col width="8.5" customWidth="1" min="11" max="11"/>
-    <col width="8.5" customWidth="1" min="12" max="12"/>
-    <col width="8.5" customWidth="1" min="13" max="13"/>
-    <col width="8.5" customWidth="1" min="14" max="14"/>
-    <col width="8.5" customWidth="1" min="15" max="15"/>
-    <col width="8.5" customWidth="1" min="16" max="16"/>
-    <col width="8.5" customWidth="1" min="17" max="17"/>
-    <col width="8.5" customWidth="1" min="18" max="18"/>
-    <col width="8.5" customWidth="1" min="19" max="19"/>
-    <col width="8.5" customWidth="1" min="20" max="20"/>
-    <col width="8.5" customWidth="1" min="21" max="21"/>
-    <col width="8.5" customWidth="1" min="22" max="22"/>
-    <col width="8.5" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="8" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,131 +545,129 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Điền chữ  x  vào MỌI buổi bạn ĐI LÀM ĐƯỢC (rảnh). Càng đăng ký nhiều buổi rảnh, càng dễ được xếp đủ ca. App sẽ tự chia cân bằng và ưu tiên người ít ca — không phải ai điền trước.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Ô XANH = đã đăng ký rảnh.  Người giữ xe do chủ quán chọn trong app.</t>
+          <t>Gõ chữ  x  vào buổi bạn RẢNH (đi làm được). Để trống = bận. Rảnh buổi nào tick buổi đó — càng nhiều càng dễ được xếp đủ ca. Chủ quán sẽ tự xếp lịch.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tên</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Vị trí</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>T2 Sáng</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>T2 Chiều</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>T2 Tối</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>T3 Sáng</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>T3 Chiều</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>T3 Tối</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>T4 Sáng</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="4" t="inlineStr">
         <is>
           <t>T4 Chiều</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>T4 Tối</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>T5 Sáng</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>T5 Chiều</t>
         </is>
       </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>T5 Tối</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>T6 Sáng</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>T6 Chiều</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>T6 Tối</t>
         </is>
       </c>
-      <c r="R4" s="6" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>T7 Sáng</t>
         </is>
       </c>
-      <c r="S4" s="6" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>T7 Chiều</t>
         </is>
       </c>
-      <c r="T4" s="6" t="inlineStr">
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>T7 Tối</t>
         </is>
       </c>
-      <c r="U4" s="5" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>CN Sáng</t>
         </is>
       </c>
-      <c r="V4" s="5" t="inlineStr">
+      <c r="V4" s="4" t="inlineStr">
         <is>
           <t>CN Chiều</t>
         </is>
       </c>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="4" t="inlineStr">
         <is>
           <t>CN Tối</t>
+        </is>
+      </c>
+      <c r="X4" s="6" t="inlineStr">
+        <is>
+          <t>Tổng rảnh</t>
         </is>
       </c>
     </row>
@@ -704,6 +695,10 @@
       <c r="U5" s="9" t="n"/>
       <c r="V5" s="9" t="n"/>
       <c r="W5" s="9" t="n"/>
+      <c r="X5" s="11">
+        <f>COUNTIF(C5:W5,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="n"/>
@@ -729,6 +724,10 @@
       <c r="U6" s="9" t="n"/>
       <c r="V6" s="9" t="n"/>
       <c r="W6" s="9" t="n"/>
+      <c r="X6" s="11">
+        <f>COUNTIF(C6:W6,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n"/>
@@ -754,6 +753,10 @@
       <c r="U7" s="9" t="n"/>
       <c r="V7" s="9" t="n"/>
       <c r="W7" s="9" t="n"/>
+      <c r="X7" s="11">
+        <f>COUNTIF(C7:W7,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n"/>
@@ -779,6 +782,10 @@
       <c r="U8" s="9" t="n"/>
       <c r="V8" s="9" t="n"/>
       <c r="W8" s="9" t="n"/>
+      <c r="X8" s="11">
+        <f>COUNTIF(C8:W8,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n"/>
@@ -804,6 +811,10 @@
       <c r="U9" s="9" t="n"/>
       <c r="V9" s="9" t="n"/>
       <c r="W9" s="9" t="n"/>
+      <c r="X9" s="11">
+        <f>COUNTIF(C9:W9,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n"/>
@@ -829,6 +840,10 @@
       <c r="U10" s="9" t="n"/>
       <c r="V10" s="9" t="n"/>
       <c r="W10" s="9" t="n"/>
+      <c r="X10" s="11">
+        <f>COUNTIF(C10:W10,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n"/>
@@ -854,6 +869,10 @@
       <c r="U11" s="9" t="n"/>
       <c r="V11" s="9" t="n"/>
       <c r="W11" s="9" t="n"/>
+      <c r="X11" s="11">
+        <f>COUNTIF(C11:W11,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n"/>
@@ -879,6 +898,10 @@
       <c r="U12" s="9" t="n"/>
       <c r="V12" s="9" t="n"/>
       <c r="W12" s="9" t="n"/>
+      <c r="X12" s="11">
+        <f>COUNTIF(C12:W12,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="n"/>
@@ -904,6 +927,10 @@
       <c r="U13" s="9" t="n"/>
       <c r="V13" s="9" t="n"/>
       <c r="W13" s="9" t="n"/>
+      <c r="X13" s="11">
+        <f>COUNTIF(C13:W13,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="n"/>
@@ -929,6 +956,10 @@
       <c r="U14" s="9" t="n"/>
       <c r="V14" s="9" t="n"/>
       <c r="W14" s="9" t="n"/>
+      <c r="X14" s="11">
+        <f>COUNTIF(C14:W14,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="n"/>
@@ -954,6 +985,10 @@
       <c r="U15" s="9" t="n"/>
       <c r="V15" s="9" t="n"/>
       <c r="W15" s="9" t="n"/>
+      <c r="X15" s="11">
+        <f>COUNTIF(C15:W15,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="n"/>
@@ -979,6 +1014,10 @@
       <c r="U16" s="9" t="n"/>
       <c r="V16" s="9" t="n"/>
       <c r="W16" s="9" t="n"/>
+      <c r="X16" s="11">
+        <f>COUNTIF(C16:W16,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="n"/>
@@ -1004,6 +1043,10 @@
       <c r="U17" s="9" t="n"/>
       <c r="V17" s="9" t="n"/>
       <c r="W17" s="9" t="n"/>
+      <c r="X17" s="11">
+        <f>COUNTIF(C17:W17,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="n"/>
@@ -1029,6 +1072,10 @@
       <c r="U18" s="9" t="n"/>
       <c r="V18" s="9" t="n"/>
       <c r="W18" s="9" t="n"/>
+      <c r="X18" s="11">
+        <f>COUNTIF(C18:W18,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="n"/>
@@ -1054,6 +1101,10 @@
       <c r="U19" s="9" t="n"/>
       <c r="V19" s="9" t="n"/>
       <c r="W19" s="9" t="n"/>
+      <c r="X19" s="11">
+        <f>COUNTIF(C19:W19,"x")</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="n"/>
@@ -1079,807 +1130,183 @@
       <c r="U20" s="9" t="n"/>
       <c r="V20" s="9" t="n"/>
       <c r="W20" s="9" t="n"/>
+      <c r="X20" s="11">
+        <f>COUNTIF(C20:W20,"x")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="10" t="n"/>
+      <c r="I21" s="9" t="n"/>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9" t="n"/>
+      <c r="L21" s="10" t="n"/>
+      <c r="M21" s="10" t="n"/>
+      <c r="N21" s="10" t="n"/>
+      <c r="O21" s="9" t="n"/>
+      <c r="P21" s="9" t="n"/>
+      <c r="Q21" s="9" t="n"/>
+      <c r="R21" s="10" t="n"/>
+      <c r="S21" s="10" t="n"/>
+      <c r="T21" s="10" t="n"/>
+      <c r="U21" s="9" t="n"/>
+      <c r="V21" s="9" t="n"/>
+      <c r="W21" s="9" t="n"/>
+      <c r="X21" s="11">
+        <f>COUNTIF(C21:W21,"x")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="10" t="n"/>
+      <c r="M22" s="10" t="n"/>
+      <c r="N22" s="10" t="n"/>
+      <c r="O22" s="9" t="n"/>
+      <c r="P22" s="9" t="n"/>
+      <c r="Q22" s="9" t="n"/>
+      <c r="R22" s="10" t="n"/>
+      <c r="S22" s="10" t="n"/>
+      <c r="T22" s="10" t="n"/>
+      <c r="U22" s="9" t="n"/>
+      <c r="V22" s="9" t="n"/>
+      <c r="W22" s="9" t="n"/>
+      <c r="X22" s="11">
+        <f>COUNTIF(C22:W22,"x")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C5:C20">
+  <conditionalFormatting sqref="C5:C22">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LOWER(C5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D5:D20">
+  <conditionalFormatting sqref="D5:D22">
     <cfRule type="expression" priority="2" dxfId="0">
       <formula>LOWER(D5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E5:E20">
+  <conditionalFormatting sqref="E5:E22">
     <cfRule type="expression" priority="3" dxfId="0">
       <formula>LOWER(E5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F5:F20">
+  <conditionalFormatting sqref="F5:F22">
     <cfRule type="expression" priority="4" dxfId="0">
       <formula>LOWER(F5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G5:G20">
+  <conditionalFormatting sqref="G5:G22">
     <cfRule type="expression" priority="5" dxfId="0">
       <formula>LOWER(G5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H20">
+  <conditionalFormatting sqref="H5:H22">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>LOWER(H5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I20">
+  <conditionalFormatting sqref="I5:I22">
     <cfRule type="expression" priority="7" dxfId="0">
       <formula>LOWER(I5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J20">
+  <conditionalFormatting sqref="J5:J22">
     <cfRule type="expression" priority="8" dxfId="0">
       <formula>LOWER(J5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K5:K20">
+  <conditionalFormatting sqref="K5:K22">
     <cfRule type="expression" priority="9" dxfId="0">
       <formula>LOWER(K5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L5:L20">
+  <conditionalFormatting sqref="L5:L22">
     <cfRule type="expression" priority="10" dxfId="0">
       <formula>LOWER(L5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M20">
+  <conditionalFormatting sqref="M5:M22">
     <cfRule type="expression" priority="11" dxfId="0">
       <formula>LOWER(M5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N20">
+  <conditionalFormatting sqref="N5:N22">
     <cfRule type="expression" priority="12" dxfId="0">
       <formula>LOWER(N5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O20">
+  <conditionalFormatting sqref="O5:O22">
     <cfRule type="expression" priority="13" dxfId="0">
       <formula>LOWER(O5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P5:P20">
+  <conditionalFormatting sqref="P5:P22">
     <cfRule type="expression" priority="14" dxfId="0">
       <formula>LOWER(P5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:Q20">
+  <conditionalFormatting sqref="Q5:Q22">
     <cfRule type="expression" priority="15" dxfId="0">
       <formula>LOWER(Q5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R5:R20">
+  <conditionalFormatting sqref="R5:R22">
     <cfRule type="expression" priority="16" dxfId="0">
       <formula>LOWER(R5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S5:S20">
+  <conditionalFormatting sqref="S5:S22">
     <cfRule type="expression" priority="17" dxfId="0">
       <formula>LOWER(S5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T5:T20">
+  <conditionalFormatting sqref="T5:T22">
     <cfRule type="expression" priority="18" dxfId="0">
       <formula>LOWER(T5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U5:U20">
+  <conditionalFormatting sqref="U5:U22">
     <cfRule type="expression" priority="19" dxfId="0">
       <formula>LOWER(U5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V5:V20">
+  <conditionalFormatting sqref="V5:V22">
     <cfRule type="expression" priority="20" dxfId="0">
       <formula>LOWER(V5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W5:W20">
+  <conditionalFormatting sqref="W5:W22">
     <cfRule type="expression" priority="21" dxfId="0">
       <formula>LOWER(W5)="x"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="B5:B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B5:B22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pha chế,Phục vụ"</formula1>
     </dataValidation>
-    <dataValidation sqref="C5:W20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C5:W22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"x"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>SỐ BẠN RẢNH MỖI BUỔI (tự cập nhật)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Số bạn đăng ký rảnh / định mức cần. Ô ĐỎ = chưa đủ người rảnh → cần thêm bạn đăng ký buổi này.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Ngày</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Buổi</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Pha chế</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Phục vụ</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C5" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!C$5:C$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D5" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C6" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D6" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C7" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D7" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C8" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D8" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C9" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D9" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C10" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D10" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C11" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D11" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C12" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D12" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C13" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D13" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C14" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D14" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C15" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D15" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C16" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D16" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C17" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D17" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C18" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D18" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>T6</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C19" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D19" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C20" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D20" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C21" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D21" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C22" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D22" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Sáng</t>
-        </is>
-      </c>
-      <c r="C23" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D23" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>Chiều</t>
-        </is>
-      </c>
-      <c r="C24" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D24" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>CN</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Tối</t>
-        </is>
-      </c>
-      <c r="C25" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&amp;"/2"</f>
-        <v/>
-      </c>
-      <c r="D25" s="8">
-        <f>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&amp;"/3"</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <conditionalFormatting sqref="C5">
-    <cfRule type="expression" priority="1" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!C$5:C$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D5">
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!C$5:C$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6">
-    <cfRule type="expression" priority="3" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!D$5:D$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6">
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!D$5:D$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C7">
-    <cfRule type="expression" priority="5" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!E$5:E$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D7">
-    <cfRule type="expression" priority="6" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!E$5:E$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8">
-    <cfRule type="expression" priority="7" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!F$5:F$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D8">
-    <cfRule type="expression" priority="8" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!F$5:F$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="expression" priority="9" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!G$5:G$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D9">
-    <cfRule type="expression" priority="10" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!G$5:G$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
-    <cfRule type="expression" priority="11" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!H$5:H$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D10">
-    <cfRule type="expression" priority="12" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!H$5:H$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
-    <cfRule type="expression" priority="13" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!I$5:I$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D11">
-    <cfRule type="expression" priority="14" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!I$5:I$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C12">
-    <cfRule type="expression" priority="15" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!J$5:J$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D12">
-    <cfRule type="expression" priority="16" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!J$5:J$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
-    <cfRule type="expression" priority="17" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!K$5:K$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D13">
-    <cfRule type="expression" priority="18" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!K$5:K$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C14">
-    <cfRule type="expression" priority="19" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!L$5:L$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D14">
-    <cfRule type="expression" priority="20" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!L$5:L$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C15">
-    <cfRule type="expression" priority="21" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!M$5:M$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D15">
-    <cfRule type="expression" priority="22" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!M$5:M$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C16">
-    <cfRule type="expression" priority="23" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!N$5:N$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D16">
-    <cfRule type="expression" priority="24" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!N$5:N$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C17">
-    <cfRule type="expression" priority="25" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!O$5:O$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D17">
-    <cfRule type="expression" priority="26" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!O$5:O$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C18">
-    <cfRule type="expression" priority="27" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!P$5:P$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D18">
-    <cfRule type="expression" priority="28" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!P$5:P$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C19">
-    <cfRule type="expression" priority="29" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!Q$5:Q$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D19">
-    <cfRule type="expression" priority="30" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!Q$5:Q$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C20">
-    <cfRule type="expression" priority="31" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!R$5:R$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D20">
-    <cfRule type="expression" priority="32" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!R$5:R$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C21">
-    <cfRule type="expression" priority="33" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!S$5:S$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D21">
-    <cfRule type="expression" priority="34" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!S$5:S$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C22">
-    <cfRule type="expression" priority="35" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!T$5:T$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D22">
-    <cfRule type="expression" priority="36" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!T$5:T$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
-    <cfRule type="expression" priority="37" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!U$5:U$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="expression" priority="38" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!U$5:U$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
-    <cfRule type="expression" priority="39" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!V$5:V$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D24">
-    <cfRule type="expression" priority="40" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!V$5:V$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C25">
-    <cfRule type="expression" priority="41" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Pha chế",'Đăng ký'!W$5:W$20,"x")&lt;2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D25">
-    <cfRule type="expression" priority="42" dxfId="1">
-      <formula>COUNTIFS('Đăng ký'!$B$5:$B$20,"Phục vụ",'Đăng ký'!W$5:W$20,"x")&lt;3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>